<commit_message>
Update CFC Fantasy League Live 2026.xlsx
</commit_message>
<xml_diff>
--- a/CFC Fantasy League Live 2026.xlsx
+++ b/CFC Fantasy League Live 2026.xlsx
@@ -466,11 +466,11 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>VS Stalwarts</t>
+          <t>Disruptors</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>20</v>
+        <v>161</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -485,17 +485,17 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>20</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Disruptors</t>
+          <t>Hilarious Hooligans</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -510,7 +510,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -535,7 +535,7 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -560,7 +560,7 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -641,11 +641,11 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Hilarious Hooligans</t>
+          <t>VS Stalwarts</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
@@ -660,7 +660,7 @@
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>-10</v>
       </c>
     </row>
   </sheetData>
@@ -674,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -707,11 +707,11 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Abhishek Sharma</t>
+          <t>Jacob Duffy</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10</v>
+        <v>121</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -723,7 +723,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>10</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -745,17 +745,17 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Jacob Duffy</t>
+          <t>Bhuvneshwar Kumar</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -767,17 +767,17 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Bhuvneshwar Kumar</t>
+          <t>Ishan Kishan</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -789,7 +789,51 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>4</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Nitish Reddy</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Abhishek Sharma</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>-5</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-5</v>
       </c>
     </row>
   </sheetData>
@@ -803,7 +847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL5"/>
+  <dimension ref="A1:AL7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -996,18 +1040,18 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Bhuvneshwar Kumar</t>
+          <t>Nitish Reddy</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>BOWL</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1044,7 +1088,7 @@
         <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
         <v>0</v>
@@ -1059,13 +1103,13 @@
         <v>0</v>
       </c>
       <c r="U2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="W2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="X2" t="n">
         <v>0</v>
@@ -1116,34 +1160,34 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Travis Head</t>
+          <t>Bhuvneshwar Kumar</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>BAT</t>
+          <t>BOWL</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -1152,7 +1196,7 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>140</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
@@ -1164,7 +1208,7 @@
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q3" t="n">
         <v>0</v>
@@ -1179,13 +1223,13 @@
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="V3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W3" t="n">
-        <v>0</v>
+        <v>7.64</v>
       </c>
       <c r="X3" t="n">
         <v>0</v>
@@ -1236,7 +1280,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Jacob Duffy</t>
+          <t>Ishan Kishan</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1247,23 +1291,23 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>BOWL</t>
+          <t>BAT</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -1272,7 +1316,7 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="M4" t="n">
         <v>0</v>
@@ -1284,7 +1328,7 @@
         <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="Q4" t="n">
         <v>0</v>
@@ -1299,13 +1343,13 @@
         <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="W4" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="X4" t="n">
         <v>0</v>
@@ -1360,7 +1404,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>-5</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -1371,7 +1415,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>10</v>
+        <v>-5</v>
       </c>
       <c r="F5" t="n">
         <v>7</v>
@@ -1392,10 +1436,10 @@
         <v>3</v>
       </c>
       <c r="L5" t="n">
-        <v>100</v>
+        <v>87.5</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>-15</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -1470,6 +1514,246 @@
         <v>0</v>
       </c>
       <c r="AL5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Travis Head</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>30</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>BAT</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>30</v>
+      </c>
+      <c r="F6" t="n">
+        <v>11</v>
+      </c>
+      <c r="G6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>4</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>122.22</v>
+      </c>
+      <c r="M6" t="n">
+        <v>15</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Jacob Duffy</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>121</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>BOWL</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
+        <v>121</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
+        <v>2</v>
+      </c>
+      <c r="T7" t="n">
+        <v>60</v>
+      </c>
+      <c r="U7" t="n">
+        <v>8</v>
+      </c>
+      <c r="V7" t="n">
+        <v>16</v>
+      </c>
+      <c r="W7" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="X7" t="n">
+        <v>20</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2496,7 +2780,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17</v>
+        <v>161</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -2510,10 +2794,10 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="G2" t="n">
-        <v>8</v>
+        <v>121</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -2573,7 +2857,7 @@
         <v>0</v>
       </c>
       <c r="AA2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AB2" t="n">
         <v>0</v>
@@ -3714,7 +3998,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -3878,7 +4162,7 @@
         <v>0</v>
       </c>
       <c r="BD4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="BE4" t="n">
         <v>0</v>
@@ -4323,7 +4607,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -4577,7 +4861,7 @@
         <v>0</v>
       </c>
       <c r="CH5" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="CI5" t="n">
         <v>0</v>
@@ -5541,7 +5825,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -6002,7 +6286,7 @@
         <v>0</v>
       </c>
       <c r="EY7" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="EZ7" t="n">
         <v>0</v>
@@ -6150,7 +6434,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>20</v>
+        <v>-10</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -6623,7 +6907,7 @@
         <v>0</v>
       </c>
       <c r="FC8" t="n">
-        <v>20</v>
+        <v>-10</v>
       </c>
       <c r="FD8" t="n">
         <v>0</v>

</xml_diff>